<commit_message>
mage: Spellsteal outranks Dragon's Breath in the dispel/CC group
Removing Dragon's Breath's spec gate had a side effect nobody asked for: at
priority 5 against Spellsteal's 6 it took Shift+X, and Spellsteal was pushed
onto a mouse thumb button. Rob, who plays the class: Spellsteal is essential
for a good player, and on Frost Dragon's Breath is a by-product of the hero
tree. Priorities swapped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/keybind_sheet/MidnightHelper_Keybinds.xlsx
+++ b/tools/keybind_sheet/MidnightHelper_Keybinds.xlsx
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Spellsteal</t>
+          <t>Dragon's Breath</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dragon's Breath, Mirror Image</t>
+          <t>Mirror Image, Spellsteal</t>
         </is>
       </c>
     </row>
@@ -5565,17 +5565,17 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+X</t>
+          <t>Ctrl+Z</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Spellsteal</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Mirror Image</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Defensive</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cauterize, Mirror Image</t>
+          <t>Cauterize, Spellsteal</t>
         </is>
       </c>
     </row>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Spellsteal</t>
+          <t>Dragon's Breath</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dragon's Breath, Mirror Image</t>
+          <t>Mirror Image, Spellsteal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the keybind cheat sheet after today's Paladin edits
Three KeybindRoles changes today -- Holy Bulwark, Rite of Sanctification, and Hand of Reckoning
widened to {66,70} -- and the sheet is meant to be rebuilt after every one of them. Both steps
through the front door, 39 specs, HTML and XLSX refreshed. The generator's own verification prints
the Prot layout and all three are in it.

Worth writing down: the sheet gives Holy Bulwark Ctrl+C while Rob's /mhautomap this morning gave it
Shift+C. Neither is broken. The sheet models the scheme with every entry that applies to the spec;
the live allocator only sees spells the character actually knows, and fewer competitors for the
overflow keys land differently. That reasoning is inferred rather than measured, but the part that
matters is not: the cheat sheet is a model of the scheme, not a mirror of one character, and a
difference against your own /mh binds is not a defect.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/keybind_sheet/MidnightHelper_Keybinds.xlsx
+++ b/tools/keybind_sheet/MidnightHelper_Keybinds.xlsx
@@ -8587,7 +8587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8756,7 +8756,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Redemption</t>
+          <t>Rite of Sanctification</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Intercession</t>
+          <t>Redemption</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -8938,46 +8938,46 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Shift+X</t>
+          <t>Shift+R</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Hammer of Justice</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Intercession</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Utility</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Shift+Z</t>
+          <t>Shift+X</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Ardent Defender</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Defensive</t>
+          <t>Hammer of Justice</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Dispel / CC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Shift+C</t>
+          <t>Shift+Z</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Divine Protection</t>
+          <t>Ardent Defender</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -8989,46 +8989,46 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Shift+V</t>
+          <t>Shift+C</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Cleanse Toxins</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Divine Protection</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Defensive</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Shift+F1</t>
+          <t>Shift+V</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Divine Toll</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Cooldown</t>
+          <t>Cleanse Toxins</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Dispel / CC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Shift+F2</t>
+          <t>Shift+F1</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Sentinel</t>
+          <t>Divine Toll</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -9040,12 +9040,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Shift+F3</t>
+          <t>Shift+F2</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Bastion of Light</t>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -9057,29 +9057,29 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+X</t>
+          <t>Shift+F3</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Repentance</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Bastion of Light</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Cooldown</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+Z</t>
+          <t>Ctrl+X</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Blessing of Protection</t>
+          <t>Blessing of Sacrifice</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -9091,12 +9091,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+C</t>
+          <t>Ctrl+Z</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Blessing of Sacrifice</t>
+          <t>Blessing of Protection</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -9108,15 +9108,32 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>Ctrl+C</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Holy Bulwark</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Defensive</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t>Ctrl+V</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Blinding Light</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>Dispel / CC</t>
         </is>
@@ -9133,7 +9150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9285,12 +9302,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Redemption</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Utility</t>
+          <t>Hand of Reckoning</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Taunt</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9319,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Intercession</t>
+          <t>Redemption</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -9484,29 +9501,29 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Shift+X</t>
+          <t>Shift+F</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Blessing of Protection</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Defensive</t>
+          <t>Intercession</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Utility</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Shift+Z</t>
+          <t>Shift+X</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Divine Protection</t>
+          <t>Blessing of Protection</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -9518,63 +9535,63 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Shift+C</t>
+          <t>Shift+Z</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Shield of Vengeance</t>
+          <t>Divine Protection</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Defensive (major)</t>
+          <t>Defensive</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Shift+V</t>
+          <t>Shift+C</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Hammer of Justice</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Shield of Vengeance</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Defensive (major)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Shift+F1</t>
+          <t>Shift+V</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Wake of Ashes</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Cooldown</t>
+          <t>Hammer of Justice</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Dispel / CC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Shift+F2</t>
+          <t>Shift+F1</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Sentinel</t>
+          <t>Wake of Ashes</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -9586,12 +9603,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Shift+F3</t>
+          <t>Shift+F2</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Divine Toll</t>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -9603,46 +9620,46 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+X</t>
+          <t>Shift+F3</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Repentance</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Dispel / CC</t>
+          <t>Divine Toll</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Cooldown</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+Z</t>
+          <t>Ctrl+X</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Blessing of Sacrifice</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>Defensive</t>
+          <t>Repentance</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Dispel / CC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+C</t>
+          <t>Ctrl+Z</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Blessing of Spellwarding</t>
+          <t>Blessing of Sacrifice</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -9654,15 +9671,32 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>Ctrl+C</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Blessing of Spellwarding</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Defensive</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t>Ctrl+V</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Blinding Light</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>Dispel / CC</t>
         </is>

</xml_diff>